<commit_message>
Redesign sample data: dense multi-row per 병록번호 pattern
53행, 20개 병록번호, 평균 2.7행/환자 — 실제 수집 환경 재현

병록번호별 행 분포:
  1행: 3개 / 2행: 7개 / 3행: 5개 / 4행: 4개 / 5행: 1개

시나리오:
  7자리 병록번호 3종류(7건), 가족 키워드 7건, 완전 중복 2건
  날짜 누락 1건, 미래날짜 1건
  F-only → P 등장 케이스, 내부코드 변경 2건, 성별 불일치 오기

README: 행수·병록번호 수·평균 업데이트

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/수집일지_샘플1.xlsx
+++ b/sample_data/수집일지_샘플1.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,57 +518,57 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>10002</v>
+        <v>10001</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P-0012</t>
+          <t>P-0011</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>12340002</t>
+          <t>12340001</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>이다라</t>
+          <t>김가나</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>F75.11</t>
+          <t>M93.05</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2024-01-16</t>
+          <t>2024-03-20</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>10003</v>
+        <v>10002</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P-0013</t>
+          <t>P-0012</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>12340003</t>
+          <t>12340002</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>박마바</t>
+          <t>이다라</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>M82.07</t>
+          <t>F75.11</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -580,650 +580,770 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>10003</v>
+        <v>10002</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>F-0031</t>
+          <t>P-0012</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>12340003</t>
+          <t>12340002</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>박마바 남편</t>
+          <t>이다라</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>M80.03</t>
+          <t>F75.11</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2024-01-16</t>
+          <t>2024-04-02</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>10004</v>
+        <v>10003</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P-0014</t>
+          <t>F-0031</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>12340004</t>
+          <t>12340003</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>최사아</t>
+          <t>박마바</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>F90.04</t>
+          <t>M82.07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2024-02-01</t>
+          <t>2024-01-20</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10005</v>
+        <v>10003</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>F-0051</t>
+          <t>F-0031</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>1234005</t>
+          <t>12340003</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>정자차</t>
+          <t>박마바</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>M01.09</t>
+          <t>M82.07</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2024-02-10</t>
+          <t>2024-03-15</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>10005</v>
+        <v>10004</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>F-0052</t>
+          <t>P-0014</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>1234005</t>
+          <t>12340004</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>정자차</t>
+          <t>최사아</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>M01.09</t>
+          <t>F90.04</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2024-02-25</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10006</v>
+        <v>10004</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P-0016</t>
+          <t>F-0041</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>12340006</t>
+          <t>12340004</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>강카타</t>
+          <t>최사아 남편</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>F55.12</t>
+          <t>M88.05</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2024-02-15</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10007</v>
+        <v>10004</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>P-0017</t>
+          <t>P-0014</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>12340007</t>
+          <t>12340004</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>조파하</t>
+          <t>최사아</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>M79.06</t>
+          <t>F90.04</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2024-02-20</t>
+          <t>2024-04-10</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10008</v>
+        <v>10005</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P-0018</t>
+          <t>F-0051</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>12340008</t>
+          <t>1234005</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>윤거너</t>
+          <t>정자차</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>F93.02</t>
+          <t>M01.09</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-02-10</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>10009</v>
+        <v>10005</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P-0019</t>
+          <t>F-0051</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>12340009</t>
+          <t>1234005</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>한서연</t>
+          <t>정자차</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>F88.08</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>M01.09</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2024-04-05</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>10010</v>
+        <v>10006</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P-0110</t>
+          <t>P-0016</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>12340010</t>
+          <t>12340006</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>임도영</t>
+          <t>강카타</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>M71.03</t>
+          <t>F55.12</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2024-03-10</t>
+          <t>2024-02-15</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>10010</v>
+        <v>10006</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>P-0110</t>
+          <t>P-0016</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>12340010</t>
+          <t>12340006</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>임도영</t>
+          <t>강카타</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>M71.03</t>
+          <t>F55.12</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2024-03-10</t>
+          <t>2024-03-28</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>10013</v>
+        <v>10006</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>P-0113</t>
+          <t>P-0016</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>1234013</t>
+          <t>12340006</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>고은지</t>
+          <t>강카타</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>F92.09</t>
+          <t>F55.12</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2024-03-20</t>
+          <t>2024-04-20</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>10015</v>
+        <v>10007</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>P-0115</t>
+          <t>P-0017</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>12340015</t>
+          <t>12340007</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>남궁민</t>
+          <t>조파하</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>M68.01</t>
+          <t>M79.06</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2099-12-01</t>
+          <t>2024-02-20</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>10016</v>
+        <v>10007</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>P-0116</t>
+          <t>F-0071</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>12340016</t>
+          <t>12340007</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>백승호</t>
+          <t>공여자</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>M90.04</t>
+          <t>F78.11</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2024-03-25</t>
+          <t>2024-02-20</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>10017</v>
+        <v>10007</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>P-0117</t>
+          <t>P-0017</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>12340017</t>
+          <t>12340007</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>신오라</t>
+          <t>조파하</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>F84.09</t>
+          <t>M79.06</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2024-03-28</t>
+          <t>2024-04-15</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>10020</v>
+        <v>10008</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>P-0120</t>
+          <t>P-0018</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>12340020</t>
+          <t>12340008</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>변바사</t>
+          <t>윤거너</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>F91.06</t>
+          <t>F93.02</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2024-03-31</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>10020</v>
+        <v>10008</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>F-0201</t>
+          <t>P-0018</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>12340020</t>
+          <t>12340008</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>공여자</t>
+          <t>윤거너</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>M89.02</t>
+          <t>F93.02</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2024-03-31</t>
+          <t>2024-04-08</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>10021</v>
+        <v>10009</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>P-0121</t>
+          <t>P-0019</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>12340021</t>
+          <t>12340009</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>오아자</t>
+          <t>한서연</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>M76.11</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>2024-04-02</t>
-        </is>
-      </c>
+          <t>F88.08</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>10022</v>
+        <v>10009</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>P-0122</t>
+          <t>P-0019</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>12340022</t>
+          <t>12340009</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>노차카</t>
+          <t>한서연</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>F83.04</t>
+          <t>F88.08</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
+          <t>2024-04-18</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>10018</v>
+        <v>10010</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>P-0118</t>
+          <t>P-0110</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>12340018</t>
+          <t>12340010</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>천도나</t>
+          <t>임도영</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>F79.08</t>
+          <t>M71.03</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>2024-03-10</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>10019</v>
+        <v>10010</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>P-0119</t>
+          <t>P-0110</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>12340019</t>
+          <t>12340010</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>황라마</t>
+          <t>임도영</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>M88.03</t>
+          <t>M71.03</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2024-04-08</t>
+          <t>2024-03-10</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>10023</v>
+        <v>10011</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>P-0123</t>
+          <t>P-0111</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>12340023</t>
+          <t>1234011</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>구타파</t>
+          <t>류민서</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>M92.08</t>
+          <t>F96.06</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2024-04-10</t>
+          <t>2024-03-22</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>10011</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>F-0111</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>1234011</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>류민서 배우자</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>M94.09</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2024-03-22</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>10012</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>P-0112</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>12340012</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>남궁민</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>M68.01</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2099-12-01</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>10013</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>P-0113</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>12340013</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>고은지</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>F92.09</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2024-04-25</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>10013</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>F-0131</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>12340013</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>태아</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2024-04-25</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>